<commit_message>
fix(payday-super-checker): address the workbook review findings
Transition confirmation ships as N, as the CLI defaults it, so the sample
is BLOCKED at that check exactly as the CLI stops without the flag.
Review Checks now flags fabricated example lines left in the register,
blocks a blank employee_id and a non-date as-at, assessment or coverage
input, and notes employee ids that differ only by capitalisation. The
item 4 lookups use EXACT in array formulas so ids stay case-sensitive as
the engine groups them; a same-table column inside EXACT in a plain
calculated column is rewritten to a this-row reference on load.
</commit_message>
<xml_diff>
--- a/packages/payday-super-checker/workbooks/payday-super-checker.xlsx
+++ b/packages/payday-super-checker/workbooks/payday-super-checker.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21ED0C93-A8DF-48A3-9022-E405BE4E7FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A45B7C-8484-47A8-8850-EA02003EFAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="232">
   <si>
     <t>Payday Super review: s 18C deadlines and the SG charge estimate</t>
   </si>
@@ -241,6 +241,12 @@
     <t>Duplicate</t>
   </si>
   <si>
+    <t>Case_variant</t>
+  </si>
+  <si>
+    <t>Sample_row</t>
+  </si>
+  <si>
     <t>EMP001</t>
   </si>
   <si>
@@ -568,15 +574,12 @@
     <t>LCR 2026/1 transition allocation reconciled and confirmed (Y/N)</t>
   </si>
   <si>
-    <t>Y</t>
+    <t>N</t>
   </si>
   <si>
     <t>Remittance-only review accepted (Y/N)</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>Holiday coverage verified until</t>
   </si>
   <si>
@@ -647,6 +650,15 @@
   </si>
   <si>
     <t>Lines assessed at a nil SG amount (nothing to assess)</t>
+  </si>
+  <si>
+    <t>As-at, assessment and coverage dates on Summary are dates</t>
+  </si>
+  <si>
+    <t>No fabricated example line from the shipped sample remains in the register</t>
+  </si>
+  <si>
+    <t>No employee ids differ only by capitalisation (treated as different people, not aligned)</t>
   </si>
   <si>
     <t>Assumptions the engine prints with every run</t>
@@ -911,8 +923,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLines" displayName="tblLines" ref="A1:BF11">
-  <tableColumns count="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLines" displayName="tblLines" ref="A1:BH11">
+  <tableColumns count="60">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="employee_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="payment_date"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="sg_amount"/>
@@ -934,7 +946,7 @@
       <calculatedColumnFormula>IF(OR(LOWER(TRIM(tblLines[[#This Row],[first_contribution_to_fund]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[first_contribution_to_fund]]&amp;""))={"","0","f","false","n","no"}),0,""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Row_problem">
-      <calculatedColumnFormula>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</calculatedColumnFormula>
+      <calculatedColumnFormula>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Guard">
       <calculatedColumnFormula>IF(OR(_xlfn.ISFORMULA(tblLines[[#This Row],[employee_id]]),_xlfn.ISFORMULA(tblLines[[#This Row],[payment_date]]),_xlfn.ISFORMULA(tblLines[[#This Row],[sg_amount]]),_xlfn.ISFORMULA(tblLines[[#This Row],[remitted_date]]),_xlfn.ISFORMULA(tblLines[[#This Row],[remitted_amount]]),_xlfn.ISFORMULA(tblLines[[#This Row],[matched_amount]]),_xlfn.ISFORMULA(tblLines[[#This Row],[fund_received_date]]),_xlfn.ISFORMULA(tblLines[[#This Row],[first_contribution_to_fund]]),_xlfn.ISFORMULA(tblLines[[#This Row],[out_of_cycle]]),_xlfn.ISFORMULA(tblLines[[#This Row],[next_standard_payday]]),_xlfn.ISFORMULA(tblLines[[#This Row],[defined_benefit]])),1,0)</calculatedColumnFormula>
@@ -949,7 +961,7 @@
       <calculatedColumnFormula>IF(tblLines[[#This Row],[Flag_ftf]]=1,WORKDAY.INTL(tblLines[[#This Row],[payment_date]],20,1,tblHolidays[date]),"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Own_due">
-      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Own_pathway">
       <calculatedColumnFormula>IF(tblLines[[#This Row],[Flag_db]]=1,"SKIP_DB",IF(tblLines[[#This Row],[Flag_ooc]]=1,IF(AND(tblLines[[#This Row],[Flag_ftf]]=1,tblLines[[#This Row],[Due_ftf]]&gt;tblLines[[#This Row],[Due_ooc]]),"EXTENDED_20BD","OUT_OF_CYCLE"),IF(tblLines[[#This Row],[Flag_ftf]]=1,"EXTENDED_20BD","USUAL_7BD")))</calculatedColumnFormula>
@@ -970,19 +982,19 @@
       <calculatedColumnFormula>IF(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),IF(tblLines[[#This Row],[Remit]]&lt;&gt;"",MIN(ROUND(tblLines[[#This Row],[remitted_amount]],2),ROUND(tblLines[[#This Row],[sg_amount]],2)),0),IF(tblLines[[#This Row],[Remit]]&lt;&gt;"",ROUND(tblLines[[#This Row],[sg_amount]],2),0))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Evidence_own">
-      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Confirmed_latest">
-      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Possible_latest">
-      <calculatedColumnFormula>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</calculatedColumnFormula>
+      <calculatedColumnFormula array="1">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Final_due">
-      <calculatedColumnFormula>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Pathway">
-      <calculatedColumnFormula>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Possible_item4">
       <calculatedColumnFormula>IF(tblLines[[#This Row],[Final_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Possible_latest]]),tblLines[[#This Row],[Possible_latest]]&gt;tblLines[[#This Row],[Final_due]]),tblLines[[#This Row],[Possible_latest]],""))</calculatedColumnFormula>
@@ -1064,6 +1076,12 @@
     </tableColumn>
     <tableColumn id="58" xr3:uid="{00000000-0010-0000-0000-00003A000000}" name="Duplicate">
       <calculatedColumnFormula>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0000-00003B000000}" name="Case_variant">
+      <calculatedColumnFormula array="1">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="60" xr3:uid="{00000000-0010-0000-0000-00003C000000}" name="Sample_row">
+      <calculatedColumnFormula>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1442,8 +1460,8 @@
     </row>
     <row r="11" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="str">
-        <f>'Review Checks'!B13</f>
-        <v>REVIEW</v>
+        <f>'Review Checks'!B16</f>
+        <v>BLOCKED</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -1469,7 +1487,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:BF11"/>
+  <dimension ref="A1:BH11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="14" width="13" customWidth="1"/>
@@ -1478,10 +1496,10 @@
     <col min="36" max="36" width="22" customWidth="1"/>
     <col min="37" max="42" width="13" customWidth="1"/>
     <col min="43" max="43" width="34" customWidth="1"/>
-    <col min="44" max="58" width="13" customWidth="1"/>
+    <col min="44" max="60" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1656,10 +1674,16 @@
       <c r="BF1" s="5" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BH1" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B2" s="7">
         <v>46212</v>
@@ -1676,14 +1700,14 @@
         <v>46219</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J2" s="7"/>
       <c r="K2" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L2" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -1698,7 +1722,7 @@
         <v>0</v>
       </c>
       <c r="O2" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P2" s="9">
@@ -1718,7 +1742,7 @@
         <v/>
       </c>
       <c r="T2" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46223</v>
       </c>
       <c r="U2" s="9" t="str">
@@ -1746,23 +1770,23 @@
         <v>612</v>
       </c>
       <c r="AA2" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>confirmed</v>
       </c>
       <c r="AB2" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB2">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC2" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC2">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD2" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46223</v>
       </c>
       <c r="AE2" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF2" s="11" t="str">
@@ -1873,10 +1897,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG2" s="9">
+        <f t="array" ref="BG2">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH2" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B3" s="7">
         <v>46212</v>
@@ -1893,14 +1925,14 @@
         <v>46238</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L3" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -1915,7 +1947,7 @@
         <v>0</v>
       </c>
       <c r="O3" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P3" s="9">
@@ -1935,7 +1967,7 @@
         <v/>
       </c>
       <c r="T3" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46223</v>
       </c>
       <c r="U3" s="9" t="str">
@@ -1963,23 +1995,23 @@
         <v>540</v>
       </c>
       <c r="AA3" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>impossible</v>
       </c>
       <c r="AB3" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB3">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC3" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC3">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD3" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46223</v>
       </c>
       <c r="AE3" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF3" s="11" t="str">
@@ -2090,10 +2122,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG3" s="9">
+        <f t="array" ref="BG3">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH3" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B4" s="7">
         <v>46212</v>
@@ -2108,14 +2148,14 @@
       <c r="F4" s="8"/>
       <c r="G4" s="7"/>
       <c r="H4" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L4" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -2130,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="O4" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P4" s="9">
@@ -2150,7 +2190,7 @@
         <v/>
       </c>
       <c r="T4" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46223</v>
       </c>
       <c r="U4" s="9" t="str">
@@ -2178,23 +2218,23 @@
         <v>318</v>
       </c>
       <c r="AA4" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>possible</v>
       </c>
       <c r="AB4" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB4">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC4" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC4">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD4" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46223</v>
       </c>
       <c r="AE4" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF4" s="11" t="str">
@@ -2305,10 +2345,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG4" s="9">
+        <f t="array" ref="BG4">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH4" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" s="7">
         <v>46212</v>
@@ -2321,14 +2369,14 @@
       <c r="F5" s="8"/>
       <c r="G5" s="7"/>
       <c r="H5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L5" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -2343,7 +2391,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P5" s="9">
@@ -2363,7 +2411,7 @@
         <v/>
       </c>
       <c r="T5" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46223</v>
       </c>
       <c r="U5" s="9" t="str">
@@ -2391,23 +2439,23 @@
         <v>0</v>
       </c>
       <c r="AA5" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>possible</v>
       </c>
       <c r="AB5" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB5">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC5" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC5">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD5" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46223</v>
       </c>
       <c r="AE5" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF5" s="11" t="str">
@@ -2518,10 +2566,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG5" s="9">
+        <f t="array" ref="BG5">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH5" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" s="7">
         <v>46212</v>
@@ -2538,14 +2594,14 @@
         <v>46239</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L6" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -2560,7 +2616,7 @@
         <v>1</v>
       </c>
       <c r="O6" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P6" s="9">
@@ -2580,7 +2636,7 @@
         <v>46241</v>
       </c>
       <c r="T6" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46241</v>
       </c>
       <c r="U6" s="9" t="str">
@@ -2608,23 +2664,23 @@
         <v>450</v>
       </c>
       <c r="AA6" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>confirmed</v>
       </c>
       <c r="AB6" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB6">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC6" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC6">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD6" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46241</v>
       </c>
       <c r="AE6" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>EXTENDED_20BD</v>
       </c>
       <c r="AF6" s="11" t="str">
@@ -2735,10 +2791,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG6" s="9">
+        <f t="array" ref="BG6">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH6" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="7">
         <v>46218</v>
@@ -2755,16 +2819,16 @@
         <v>46234</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J7" s="7">
         <v>46226</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L7" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -2779,7 +2843,7 @@
         <v>0</v>
       </c>
       <c r="O7" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P7" s="9">
@@ -2799,7 +2863,7 @@
         <v/>
       </c>
       <c r="T7" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46238</v>
       </c>
       <c r="U7" s="9" t="str">
@@ -2827,23 +2891,23 @@
         <v>120</v>
       </c>
       <c r="AA7" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>confirmed</v>
       </c>
       <c r="AB7" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB7">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC7" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC7">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD7" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46238</v>
       </c>
       <c r="AE7" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>OUT_OF_CYCLE</v>
       </c>
       <c r="AF7" s="11" t="str">
@@ -2954,10 +3018,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG7" s="9">
+        <f t="array" ref="BG7">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH7" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B8" s="7">
         <v>46212</v>
@@ -2974,14 +3046,14 @@
         <v>46216</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J8" s="7"/>
       <c r="K8" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -2996,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P8" s="9">
@@ -3015,9 +3087,9 @@
         <f>IF(tblLines[[#This Row],[Flag_ftf]]=1,WORKDAY.INTL(tblLines[[#This Row],[payment_date]],20,1,tblHolidays[date]),"")</f>
         <v/>
       </c>
-      <c r="T8" s="11" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
-        <v/>
+      <c r="T8" s="11">
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <v>0</v>
       </c>
       <c r="U8" s="9" t="str">
         <f>IF(tblLines[[#This Row],[Flag_db]]=1,"SKIP_DB",IF(tblLines[[#This Row],[Flag_ooc]]=1,IF(AND(tblLines[[#This Row],[Flag_ftf]]=1,tblLines[[#This Row],[Due_ftf]]&gt;tblLines[[#This Row],[Due_ooc]]),"EXTENDED_20BD","OUT_OF_CYCLE"),IF(tblLines[[#This Row],[Flag_ftf]]=1,"EXTENDED_20BD","USUAL_7BD")))</f>
@@ -3044,23 +3116,23 @@
         <v>900</v>
       </c>
       <c r="AA8" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>impossible</v>
       </c>
       <c r="AB8" s="11" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB8">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v/>
       </c>
       <c r="AC8" s="11" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC8">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v/>
       </c>
       <c r="AD8" s="11" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v/>
       </c>
       <c r="AE8" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>SKIP_DB</v>
       </c>
       <c r="AF8" s="11" t="str">
@@ -3171,10 +3243,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG8" s="9">
+        <f t="array" ref="BG8">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH8" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B9" s="7">
         <v>46226</v>
@@ -3191,14 +3271,14 @@
         <v>46240</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J9" s="7"/>
       <c r="K9" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -3213,7 +3293,7 @@
         <v>0</v>
       </c>
       <c r="O9" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P9" s="9">
@@ -3233,7 +3313,7 @@
         <v/>
       </c>
       <c r="T9" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46238</v>
       </c>
       <c r="U9" s="9" t="str">
@@ -3261,23 +3341,23 @@
         <v>612</v>
       </c>
       <c r="AA9" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>impossible</v>
       </c>
       <c r="AB9" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB9">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>46223</v>
       </c>
       <c r="AC9" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC9">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>46223</v>
       </c>
       <c r="AD9" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46238</v>
       </c>
       <c r="AE9" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF9" s="11" t="str">
@@ -3388,10 +3468,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG9" s="9">
+        <f t="array" ref="BG9">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH9" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B10" s="7">
         <v>46226</v>
@@ -3408,14 +3496,14 @@
         <v>46233</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J10" s="7"/>
       <c r="K10" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -3430,7 +3518,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P10" s="9">
@@ -3450,7 +3538,7 @@
         <v/>
       </c>
       <c r="T10" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46238</v>
       </c>
       <c r="U10" s="9" t="str">
@@ -3478,23 +3566,23 @@
         <v>540</v>
       </c>
       <c r="AA10" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>confirmed</v>
       </c>
       <c r="AB10" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB10">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AC10" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC10">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>0</v>
       </c>
       <c r="AD10" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46238</v>
       </c>
       <c r="AE10" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>USUAL_7BD</v>
       </c>
       <c r="AF10" s="11" t="str">
@@ -3605,10 +3693,18 @@
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:58" x14ac:dyDescent="0.25">
+      <c r="BG10" s="9">
+        <f t="array" ref="BG10">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH10" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B11" s="7">
         <v>46226</v>
@@ -3625,14 +3721,14 @@
         <v>46240</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"1","t","true","y","yes"}),1,IF(OR(LOWER(TRIM(tblLines[[#This Row],[defined_benefit]]&amp;""))={"","0","f","false","n","no"}),0,""))</f>
@@ -3647,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="9" t="str">
-        <f>TRIM(IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
+        <f>TRIM(IF(TRIM(tblLines[[#This Row],[employee_id]]&amp;"")="","employee_id ","")&amp;IF(OR(AND(tblLines[[#This Row],[payment_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),AND(tblLines[[#This Row],[remitted_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),AND(tblLines[[#This Row],[fund_received_date]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[fund_received_date]]))),AND(tblLines[[#This Row],[next_standard_payday]]&lt;&gt;"",NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]])))),"date ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[payment_date]])),"payment_date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[payment_date]]&lt;DATE(2026,7,1)),"pre-1-Jul-2026 ","")&amp;IF(OR(AND(tblLines[[#This Row],[sg_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),tblLines[[#This Row],[sg_amount]]&lt;0)),AND(tblLines[[#This Row],[remitted_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]])),tblLines[[#This Row],[remitted_amount]]&lt;0)),AND(tblLines[[#This Row],[matched_amount]]&lt;&gt;"",OR(NOT(ISNUMBER(tblLines[[#This Row],[matched_amount]])),tblLines[[#This Row],[matched_amount]]&lt;0))),"amount ","")&amp;IF(NOT(ISNUMBER(tblLines[[#This Row],[sg_amount]])),"sg_amount ","")&amp;IF(OR(tblLines[[#This Row],[Flag_ftf]]="",tblLines[[#This Row],[Flag_ooc]]="",tblLines[[#This Row],[Flag_db]]=""),"yes/no ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"remitted_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_amount]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_date]]))),"remitted_amount-needs-date ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&gt;tblLines[[#This Row],[sg_amount]]),"matched_amount&gt;sg ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[remitted_amount]]),tblLines[[#This Row],[remitted_amount]]&gt;tblLines[[#This Row],[matched_amount]]),"remitted_amount&gt;matched ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[matched_amount]]),ISNUMBER(tblLines[[#This Row],[sg_amount]]),tblLines[[#This Row],[matched_amount]]&lt;tblLines[[#This Row],[sg_amount]],ISNUMBER(tblLines[[#This Row],[remitted_date]]),NOT(ISNUMBER(tblLines[[#This Row],[remitted_amount]]))),"partial-match-needs-remitted_amount ","")&amp;IF(AND(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[remitted_date]]),"receipt-before-remittance ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,NOT(ISNUMBER(tblLines[[#This Row],[next_standard_payday]]))),"out_of_cycle-needs-next_standard_payday ","")&amp;IF(AND(tblLines[[#This Row],[Flag_ooc]]=1,ISNUMBER(tblLines[[#This Row],[next_standard_payday]]),ISNUMBER(tblLines[[#This Row],[payment_date]]),tblLines[[#This Row],[next_standard_payday]]&lt;=tblLines[[#This Row],[payment_date]]),"next_standard_payday-not-after-payday ",""))</f>
         <v/>
       </c>
       <c r="P11" s="9">
@@ -3667,7 +3763,7 @@
         <v/>
       </c>
       <c r="T11" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),"",IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
+        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,NOT(ISNUMBER(tblLines[[#This Row],[payment_date]]))),0,IF(OR(tblLines[[#This Row],[Flag_ooc]]=1,tblLines[[#This Row],[Flag_ftf]]=1),MAX(tblLines[[#This Row],[Due_ooc]],tblLines[[#This Row],[Due_ftf]]),WORKDAY.INTL(tblLines[[#This Row],[payment_date]],7,1,tblHolidays[date])))</f>
         <v>46238</v>
       </c>
       <c r="U11" s="9" t="str">
@@ -3695,23 +3791,23 @@
         <v>450</v>
       </c>
       <c r="AA11" s="9" t="str">
-        <f>IF(OR(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
+        <f>IF(OR(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[sg_amount]]&lt;=0,tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Cap]]&lt;=0),"impossible",IF(ISNUMBER(tblLines[[#This Row],[fund_received_date]]),IF(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[Earliest_prepay]],"impossible",IF(tblLines[[#This Row],[fund_received_date]]&lt;=Summary!$B$2,IF(OR(tblLines[[#This Row],[fund_received_date]]&lt;tblLines[[#This Row],[payment_date]],tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]]),"confirmed",IF(tblLines[[#This Row],[fund_received_date]]&gt;tblLines[[#This Row],[Own_due]],"impossible","possible")),IF(tblLines[[#This Row],[fund_received_date]]&lt;=tblLines[[#This Row],[Own_due]],"possible","impossible"))),IF(AND(ISNUMBER(tblLines[[#This Row],[remitted_date]]),tblLines[[#This Row],[remitted_date]]&gt;tblLines[[#This Row],[Own_due]]),"impossible","possible")))</f>
         <v>impossible</v>
       </c>
       <c r="AB11" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"confirmed"))</f>
+        <f t="array" ref="AB11">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]="confirmed")*tblLines[Own_due])))</f>
         <v>46241</v>
       </c>
       <c r="AC11" s="11">
-        <f>IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=""),"",_xlfn.MAXIFS(tblLines[Own_due],tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],"&lt;"&amp;tblLines[[#This Row],[payment_date]],tblLines[Evidence_own],"&lt;&gt;impossible"))</f>
+        <f t="array" ref="AC11">IF(OR(tblLines[[#This Row],[Flag_db]]=1,tblLines[[#This Row],[Own_due]]=0),"",SUMPRODUCT(MAX(EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])*(tblLines[payment_date]&lt;tblLines[[#This Row],[payment_date]])*(tblLines[Evidence_own]&lt;&gt;"impossible")*tblLines[Own_due])))</f>
         <v>46241</v>
       </c>
       <c r="AD11" s="11">
-        <f>IF(tblLines[[#This Row],[Own_due]]="","",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,"",IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),tblLines[[#This Row],[Confirmed_latest]],tblLines[[#This Row],[Own_due]]))</f>
         <v>46241</v>
       </c>
       <c r="AE11" s="9" t="str">
-        <f>IF(tblLines[[#This Row],[Own_due]]="",tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
+        <f>IF(tblLines[[#This Row],[Own_due]]=0,tblLines[[#This Row],[Own_pathway]],IF(AND(ISNUMBER(tblLines[[#This Row],[Confirmed_latest]]),tblLines[[#This Row],[Confirmed_latest]]&gt;tblLines[[#This Row],[Own_due]]),"ITEM4_ALIGNED",tblLines[[#This Row],[Own_pathway]]))</f>
         <v>ITEM4_ALIGNED</v>
       </c>
       <c r="AF11" s="11" t="str">
@@ -3821,6 +3917,14 @@
       <c r="BF11" s="9">
         <f>IF(COUNTIFS(tblLines[employee_id],tblLines[[#This Row],[employee_id]],tblLines[payment_date],tblLines[[#This Row],[payment_date]],tblLines[sg_amount],tblLines[[#This Row],[sg_amount]],tblLines[remitted_date],tblLines[[#This Row],[remitted_date]]&amp;"",tblLines[fund_received_date],tblLines[[#This Row],[fund_received_date]]&amp;"")&gt;1,1,0)</f>
         <v>0</v>
+      </c>
+      <c r="BG11" s="9">
+        <f t="array" ref="BG11">IF(COUNTIF(tblLines[employee_id],tblLines[[#This Row],[employee_id]])&gt;SUMPRODUCT(--EXACT(tblLines[employee_id],tblLines[[#This Row],[employee_id]])),1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="BH11" s="9">
+        <f>IF(AND(ISNUMBER(MATCH(tblLines[[#This Row],[employee_id]],{"EMP001","EMP002","EMP003","EMP004","EMP005","EMP006","EMP007","EMP001","EMP002","EMP005"},0)),ISNUMBER(MATCH(tblLines[[#This Row],[payment_date]],{46212,46212,46212,46212,46212,46218,46212,46226,46226,46226},0))),1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3846,30 +3950,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -3883,10 +3987,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -3900,10 +4004,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -3917,10 +4021,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -3934,13 +4038,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -3954,10 +4058,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -3971,10 +4075,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -3988,13 +4092,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -4008,10 +4112,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -4025,13 +4129,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D11">
         <v>0</v>
@@ -4045,13 +4149,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -4065,13 +4169,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -4085,13 +4189,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -4105,13 +4209,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -4125,10 +4229,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -4142,13 +4246,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -4162,10 +4266,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -4179,10 +4283,10 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -4196,10 +4300,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B20" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -4213,13 +4317,13 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B21" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -4233,13 +4337,13 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -4253,10 +4357,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -4270,10 +4374,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B24" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D24">
         <v>0</v>
@@ -4287,13 +4391,13 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -4307,10 +4411,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B26" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -4324,10 +4428,10 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -4359,13 +4463,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -4373,10 +4477,10 @@
         <v>46023</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -4384,10 +4488,10 @@
         <v>46048</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -4395,10 +4499,10 @@
         <v>46083</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -4406,10 +4510,10 @@
         <v>46090</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -4417,10 +4521,10 @@
         <v>46115</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4428,10 +4532,10 @@
         <v>46116</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4439,10 +4543,10 @@
         <v>46117</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4450,10 +4554,10 @@
         <v>46118</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -4461,10 +4565,10 @@
         <v>46137</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -4472,10 +4576,10 @@
         <v>46139</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -4483,10 +4587,10 @@
         <v>46146</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -4494,10 +4598,10 @@
         <v>46174</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -4505,10 +4609,10 @@
         <v>46181</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -4516,10 +4620,10 @@
         <v>46237</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4527,10 +4631,10 @@
         <v>46290</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -4538,10 +4642,10 @@
         <v>46300</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -4549,10 +4653,10 @@
         <v>46381</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -4560,10 +4664,10 @@
         <v>46382</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -4571,10 +4675,10 @@
         <v>46384</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4582,10 +4686,10 @@
         <v>46388</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -4593,10 +4697,10 @@
         <v>46413</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -4604,10 +4708,10 @@
         <v>46447</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -4615,10 +4719,10 @@
         <v>46454</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -4626,10 +4730,10 @@
         <v>46472</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -4637,10 +4741,10 @@
         <v>46473</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -4648,10 +4752,10 @@
         <v>46474</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -4659,10 +4763,10 @@
         <v>46475</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -4670,10 +4774,10 @@
         <v>46502</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -4681,10 +4785,10 @@
         <v>46503</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -4692,10 +4796,10 @@
         <v>46510</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -4703,10 +4807,10 @@
         <v>46538</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -4714,10 +4818,10 @@
         <v>46545</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -4725,10 +4829,10 @@
         <v>46552</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C34" s="12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -4736,10 +4840,10 @@
         <v>46601</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -4747,10 +4851,10 @@
         <v>46664</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -4758,10 +4862,10 @@
         <v>46746</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -4769,10 +4873,10 @@
         <v>46747</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -4780,10 +4884,10 @@
         <v>46748</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -4791,20 +4895,20 @@
         <v>46749</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -4825,22 +4929,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -4857,10 +4961,10 @@
         <v>365</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -4877,10 +4981,10 @@
         <v>365</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -4897,7 +5001,7 @@
         <v>365</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F4" s="12"/>
     </row>
@@ -4915,7 +5019,7 @@
         <v>365</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F5" s="12"/>
     </row>
@@ -4933,7 +5037,7 @@
         <v>366</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F6" s="12"/>
     </row>
@@ -4951,7 +5055,7 @@
         <v>365</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F7" s="12"/>
     </row>
@@ -4969,13 +5073,13 @@
         <v>365</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F8" s="12"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -4997,13 +5101,13 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B2" s="13">
         <v>46244</v>
@@ -5011,21 +5115,21 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B3" s="13"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>178</v>
@@ -5033,7 +5137,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B6" s="13">
         <v>46630</v>
@@ -5041,7 +5145,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" s="11">
         <f>_xlfn.MAXIFS(tblGic[to],tblGic[basis],"known")</f>
@@ -5050,13 +5154,13 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B9" s="5"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B10" s="9">
         <f>COUNTIF(tblLines[Verdict],"ON_TIME")</f>
@@ -5065,7 +5169,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTIF(tblLines[Verdict],"AT_RISK")</f>
@@ -5074,7 +5178,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B12" s="9">
         <f>COUNTIF(tblLines[Verdict],"LATE")</f>
@@ -5083,7 +5187,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B13" s="9">
         <f>COUNTIF(tblLines[Verdict],"UNPAID")</f>
@@ -5092,7 +5196,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B14" s="9">
         <f>COUNTIF(tblLines[Verdict],"UNKNOWN")</f>
@@ -5101,7 +5205,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B15" s="9">
         <f>COUNTIF(tblLines[Verdict],"SKIPPED")</f>
@@ -5110,7 +5214,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B16" s="9">
         <f>SUM(tblLines[Exposed])</f>
@@ -5119,7 +5223,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B17" s="10">
         <f>ROUND(SUM(tblLines[Shortfall_r]),2)</f>
@@ -5128,7 +5232,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B18" s="10">
         <f>ROUND(SUM(tblLines[NEC_r]),2)</f>
@@ -5137,7 +5241,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B19" s="10">
         <f>ROUND(SUM(tblLines[SGC_low]),2)</f>
@@ -5146,7 +5250,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B20" s="10">
         <f>ROUND(SUM(tblLines[SGC_high]),2)</f>
@@ -5155,7 +5259,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B21" s="9">
         <f>SUMPRODUCT(--(tblLines[Unassessable_between]&lt;&gt;""))</f>
@@ -5164,7 +5268,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B22" s="9" t="str">
         <f>IF(AND(SUM(tblLines[Assessable])&gt;0,SUMPRODUCT(tblLines[Assessable]*tblLines[Receipt_established])=0),"YES","NO")</f>
@@ -5176,8 +5280,8 @@
         <v>7</v>
       </c>
       <c r="B24" s="15" t="str">
-        <f>'Review Checks'!B13</f>
-        <v>REVIEW</v>
+        <f>'Review Checks'!B16</f>
+        <v>BLOCKED</v>
       </c>
     </row>
   </sheetData>
@@ -5193,9 +5297,15 @@
       <formula>"PASS"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation type="list" sqref="B4:B5" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" sqref="B2 B6" xr:uid="{00000000-0002-0000-0500-000002000000}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" sqref="B3" xr:uid="{00000000-0002-0000-0500-000003000000}">
+      <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5204,7 +5314,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
@@ -5215,21 +5325,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B2" s="9" t="str">
         <f>IF(C2=0,"PASS","BLOCKED")</f>
@@ -5246,7 +5356,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B3" s="9" t="str">
         <f>IF(C3=0,"PASS","BLOCKED")</f>
@@ -5263,11 +5373,11 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B4" s="9" t="str">
         <f>IF(OR(C4=0,Summary!$B$4="Y"),"PASS","BLOCKED")</f>
-        <v>PASS</v>
+        <v>BLOCKED</v>
       </c>
       <c r="C4" s="9">
         <f>SUM(tblLines[Transition_row])</f>
@@ -5280,7 +5390,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B5" s="9" t="str">
         <f>IF(C5=0,"PASS","REVIEW")</f>
@@ -5297,7 +5407,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B6" s="9" t="str">
         <f>IF(C6=0,"PASS","REVIEW")</f>
@@ -5314,7 +5424,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B7" s="9" t="str">
         <f>IF(OR(Summary!B22="NO",Summary!$B$5="Y"),"PASS","REVIEW")</f>
@@ -5328,7 +5438,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B8" s="9" t="str">
         <f>IF(C8=0,"PASS","NOTE")</f>
@@ -5345,7 +5455,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B9" s="9" t="str">
         <f>IF(C9=0,"PASS","NOTE")</f>
@@ -5362,7 +5472,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B10" s="9" t="str">
         <f>IF(C10=0,"PASS","NOTE")</f>
@@ -5379,7 +5489,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B11" s="9" t="str">
         <f>IF(C11=0,"PASS","NOTE")</f>
@@ -5394,53 +5504,101 @@
         <v/>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="9" t="str">
+        <f>IF(AND(ISNUMBER(Summary!$B$2),OR(Summary!$B$3="",ISNUMBER(Summary!$B$3)),ISNUMBER(Summary!$B$6)),"PASS","BLOCKED")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C12" s="9">
+        <f>Summary!$B$2</f>
+        <v>46244</v>
+      </c>
+      <c r="D12" s="9"/>
+    </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="9" t="str">
+        <f>IF(C13=0,"PASS","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="C13" s="9">
+        <f>SUM(tblLines[Sample_row])</f>
+        <v>10</v>
+      </c>
+      <c r="D13" s="9" t="str">
+        <f t="array" ref="D13">IF(C13=0,"",INDEX(tblLines[employee_id],SUMPRODUCT(MAX((tblLines[Sample_row]=1)*(ROW(tblLines[employee_id])-1)))))</f>
+        <v>EMP005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B14" s="9" t="str">
+        <f>IF(C14=0,"PASS","NOTE")</f>
+        <v>PASS</v>
+      </c>
+      <c r="C14" s="9">
+        <f>SUM(tblLines[Case_variant])</f>
+        <v>0</v>
+      </c>
+      <c r="D14" s="9" t="str">
+        <f t="array" ref="D14">IF(C14=0,"",INDEX(tblLines[employee_id],SUMPRODUCT(MAX((tblLines[Case_variant]=1)*(ROW(tblLines[employee_id])-1)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="15" t="str">
-        <f>IF(COUNTIF(B2:B11,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B11,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
-        <v>REVIEW</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
-        <v>206</v>
+      <c r="B16" s="15" t="str">
+        <f>IF(COUNTIF(B2:B14,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B14,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
+        <v>BLOCKED</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="16" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <conditionalFormatting sqref="B2:B13">
+  <conditionalFormatting sqref="B2:B16">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"BLOCKED"</formula>
     </cfRule>
@@ -5466,74 +5624,74 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B5" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B6" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B7" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B9" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>